<commit_message>
Store starting formula results so previews show totals; date samples before bid day
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TUXTZtKaZKWmVHGJU2Z7sN
</commit_message>
<xml_diff>
--- a/samples/Riverside Clinic TI - Electrical leveling (sample).xlsx
+++ b/samples/Riverside Clinic TI - Electrical leveling (sample).xlsx
@@ -984,7 +984,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bids due 2026-11-04</t>
+          <t>Bids due 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1054,23 +1054,23 @@
       </c>
       <c r="E5" s="4">
         <f>SUM(Leveling!E5:E65)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F5" s="4">
         <f>IF(D5="","",D5+E5)</f>
-        <v/>
+        <v>186400</v>
       </c>
       <c r="G5" s="3">
         <f>COUNTIFS(Leveling!D5:D65,"Excluded",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="H5" s="3">
         <f>COUNTIFS(Leveling!D5:D65,"Not mentioned",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="I5" s="3">
         <f>COUNTIFS(Leveling!D5:D65,"Qualified",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -1092,23 +1092,23 @@
       </c>
       <c r="E6" s="4">
         <f>SUM(Leveling!G5:G65)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F6" s="4">
         <f>IF(D6="","",D6+E6)</f>
-        <v/>
+        <v>171250</v>
       </c>
       <c r="G6" s="3">
         <f>COUNTIFS(Leveling!F5:F65,"Excluded",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="H6" s="3">
         <f>COUNTIFS(Leveling!F5:F65,"Not mentioned",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="I6" s="3">
         <f>COUNTIFS(Leveling!F5:F65,"Qualified",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C7" s="3" t="n"/>
@@ -1128,23 +1128,23 @@
       </c>
       <c r="E7" s="4">
         <f>SUM(Leveling!I5:I65)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F7" s="4">
         <f>IF(D7="","",D7+E7)</f>
-        <v/>
+        <v>198900</v>
       </c>
       <c r="G7" s="3">
         <f>COUNTIFS(Leveling!H5:H65,"Excluded",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="H7" s="3">
         <f>COUNTIFS(Leveling!H5:H65,"Not mentioned",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>16</v>
       </c>
       <c r="I7" s="3">
         <f>COUNTIFS(Leveling!H5:H65,"Qualified",Leveling!$C$5:$C$65,"Y")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Exclusion 16 says any work not listed is excluded. Can you confirm you priced everything on E0.1-E4.2?</t>
+          <t>Exclusion 16 says any work not listed is excluded. Can you confirm you priced everything on E0.1-E4.2 dated 9/15/26?</t>
         </is>
       </c>
     </row>

</xml_diff>